<commit_message>
docs: Add existing and proposed schemas for Email & SMS Management
- Created EMAIL_SMS_SCHEMA_EXISTING.svg to represent the current state of the notification core, including trigger_events, notification_templates, notification_logs, allowed_from_domains, and enums.
- Introduced EMAIL_SMS_SCHEMA_PROPOSED.svg to outline the proposed changes, which include new scheduling capabilities, additional tables (notification_schedules and notification_schedule_occurrences), and new enums (NotificationScheduleKind, NotificationStopCondition, OccurrenceStatus).
- Updated existing entities to include new fields for scheduling support and clarified relationships between tables.
</commit_message>
<xml_diff>
--- a/EMAIL_SMS_Consolidated_Template_List.xlsx
+++ b/EMAIL_SMS_Consolidated_Template_List.xlsx
@@ -85,7 +85,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -107,11 +107,55 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -141,6 +185,8 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -555,11 +601,11 @@
           <t>PART A — 40 CLIENT-LIST ITEMS</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n"/>
-      <c r="D2" s="3" t="n"/>
-      <c r="E2" s="3" t="n"/>
-      <c r="F2" s="3" t="n"/>
+      <c r="B2" s="13" t="n"/>
+      <c r="C2" s="13" t="n"/>
+      <c r="D2" s="13" t="n"/>
+      <c r="E2" s="13" t="n"/>
+      <c r="F2" s="14" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
@@ -1767,11 +1813,11 @@
           <t>PART B — 12 SYSTEM-ONLY IMPLEMENTED TEMPLATES</t>
         </is>
       </c>
-      <c r="B43" s="3" t="n"/>
-      <c r="C43" s="3" t="n"/>
-      <c r="D43" s="3" t="n"/>
-      <c r="E43" s="3" t="n"/>
-      <c r="F43" s="3" t="n"/>
+      <c r="B43" s="13" t="n"/>
+      <c r="C43" s="13" t="n"/>
+      <c r="D43" s="13" t="n"/>
+      <c r="E43" s="13" t="n"/>
+      <c r="F43" s="14" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="4" t="n">
@@ -2039,7 +2085,7 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>REC (cron)</t>
+          <t>system cron (not in new schedule model; is_schedulable=false)</t>
         </is>
       </c>
     </row>
@@ -2069,7 +2115,7 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>REC (cron)</t>
+          <t>system cron (not in new schedule model; is_schedulable=false)</t>
         </is>
       </c>
     </row>
@@ -2099,7 +2145,7 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>REC (cron)</t>
+          <t>system cron (not in new schedule model; is_schedulable=false)</t>
         </is>
       </c>
     </row>
@@ -2129,7 +2175,7 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>REC (cron)</t>
+          <t>system cron (not in new schedule model; is_schedulable=false)</t>
         </is>
       </c>
     </row>
@@ -2148,7 +2194,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B38"/>
+  <dimension ref="A1:B41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -2256,7 +2302,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Transactional / instant — sent immediately on its trigger; not schedulable. (cron) = currently on a fixed system cron, not admin-configurable.</t>
+          <t>Transactional / instant — sent immediately on its trigger; not schedulable. "system cron" = an existing fixed background-worker cron (is_schedulable=false), NOT a RECURRING notification_schedules row and not admin-configurable.</t>
         </is>
       </c>
     </row>
@@ -2315,134 +2361,160 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>Runtime boundary (this build)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>SMS rows</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Occurrence materializes but dispatch is SKIPPED until an SMS provider is integrated (Known-Issue #2).</t>
+        </is>
+      </c>
+    </row>
     <row r="21">
-      <c r="A21" s="11" t="inlineStr">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Token-recipient rows</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Author-able, but occurrences DEFER/SKIP until Dynamic Recipient Resolution lands (Known-Issue #3); only fixed or anchor-row-column recipients dispatch now.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24">
+      <c r="A24" s="11" t="inlineStr">
         <is>
           <t>Reconciliation</t>
         </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Client-list items (Part A)</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  of which Both (B) — client rows</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  of which Client-only (C)</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>35</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>System-only implemented (Part B, S)</t>
+          <t>Client-list items (Part A)</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>12</v>
+        <v>40</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="12" t="inlineStr">
-        <is>
-          <t>TOTAL DISTINCT TEMPLATES</t>
-        </is>
-      </c>
-      <c r="B26" s="12" t="n">
-        <v>52</v>
+      <c r="A26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  of which Both (B) — client rows</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr"/>
-      <c r="B27" t="inlineStr"/>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  of which Client-only (C)</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>35</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Formula: 40 + (18 implemented - 6 overlap) = 40 + 12</t>
+          <t>System-only implemented (Part B, S)</t>
         </is>
       </c>
       <c r="B28" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="12" t="inlineStr">
+        <is>
+          <t>TOTAL DISTINCT TEMPLATES</t>
+        </is>
+      </c>
+      <c r="B29" s="12" t="n">
         <v>52</v>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" t="inlineStr"/>
-      <c r="B29" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>By channel — Email</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
-        <v>48</v>
-      </c>
-    </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>By channel — SMS</t>
+          <t>Formula: 40 + (18 implemented - 6 overlap) = 40 + 12</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>4</v>
-      </c>
-    </row>
+        <v>52</v>
+      </c>
+    </row>
+    <row r="32"/>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Note: the 6 implemented 'Both' templates collapse into 5 client rows — admin (forgot_password) and</t>
-        </is>
+          <t>By channel — Email</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>48</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>exhibitor (exhibitor_forgot_password) password-reset are two separate templates under the single</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>client 'Password Reset Request' row. Split them and the distinct count becomes 53.</t>
-        </is>
-      </c>
-    </row>
+          <t>By channel — SMS</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="35"/>
     <row r="36">
-      <c r="A36" t="inlineStr"/>
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Note: the 6 implemented 'Both' templates collapse into 5 client rows — admin (forgot_password) and</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Source: ONLY_Auto_Email_Notification_Triggers.xlsx ('Auto Emails' tab, 40 line items) +</t>
+          <t>exhibitor (exhibitor_forgot_password) password-reset are two separate templates under the single</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
+        <is>
+          <t>client 'Password Reset Request' row. Split them and the distinct count becomes 53.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39"/>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Source: ONLY_Auto_Email_Notification_Triggers.xlsx ('Auto Emails' tab, 40 line items) +</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
         <is>
           <t>admin-backend-api/src/database/seeds/notification-template.seeder.ts (18 seeded bodies).</t>
         </is>

</xml_diff>